<commit_message>
Added day-wise and subject-wise Excel export, improved PDF layout and download system
</commit_message>
<xml_diff>
--- a/Monday_Class_Timetable.xlsx
+++ b/Monday_Class_Timetable.xlsx
@@ -1037,17 +1037,17 @@
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>GENERAL SCIENCE (TABUSSUM)</t>
+          <t>GENERAL SCIENCE (FARHANA IMRAN)</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>GP (BUSHRA JAMSHED)</t>
+          <t>AI (AI TEACHER)</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>SINDHI (GHAZALA)</t>
+          <t>Geography (IRUM BATOOL)</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
@@ -1230,12 +1230,12 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
+          <t>COMPUTER (IRUM NAZ)</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
           <t>S.ST (NADIA AMIR)</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>COMPUTER (IRUM NAZ)</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
@@ -1329,7 +1329,7 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>LIBRARY (LIB TEACHER)</t>
+          <t>BIOLOGY (TABUSSUM)</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
@@ -1433,7 +1433,7 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>ENGLISH (AMINA NADEEM)</t>
+          <t>ENGLISH (IRUM BATOOL)</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
@@ -1844,12 +1844,12 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>SINDHI-X (GHAZALA)</t>
+          <t>SINDHI-X (MARVI)</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>ENGLISH (IRUM BATOOL)</t>
+          <t>ENGLISH (AMINA NADEEM)</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">

</xml_diff>